<commit_message>
feat: estruturar trasnformação do contas_recebidas
</commit_message>
<xml_diff>
--- a/stage/transform/files/reference/dim_conta_cc.xlsx
+++ b/stage/transform/files/reference/dim_conta_cc.xlsx
@@ -12,6 +12,9 @@
     <sheet name="tipos_documento" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="instrucoes" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">conta_cc!$A$1:$K$306</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -22,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1672" uniqueCount="753">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1673" uniqueCount="753">
   <si>
     <t xml:space="preserve">empresa_cod</t>
   </si>
@@ -2307,7 +2310,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2349,6 +2352,11 @@
       <name val="Courier New"/>
       <family val="3"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -2459,7 +2467,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2492,7 +2500,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2500,7 +2512,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2516,7 +2528,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2533,11 +2545,27 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="6">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF595959"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -2552,7 +2580,15 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
+          <fgColor rgb="FF1F4E79"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF375623"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -2619,6 +2655,10 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2902,7 +2942,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="n">
         <v>17</v>
       </c>
@@ -2952,7 +2992,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="n">
         <v>21</v>
       </c>
@@ -2977,7 +3017,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="n">
         <v>22</v>
       </c>
@@ -3002,7 +3042,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="n">
         <v>20</v>
       </c>
@@ -3027,7 +3067,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="n">
         <v>21</v>
       </c>
@@ -3052,7 +3092,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="n">
         <v>20</v>
       </c>
@@ -3102,7 +3142,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="n">
         <v>18</v>
       </c>
@@ -3127,7 +3167,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="n">
         <v>1</v>
       </c>
@@ -3158,7 +3198,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="n">
         <v>19</v>
       </c>
@@ -3183,7 +3223,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="n">
         <v>1</v>
       </c>
@@ -3208,7 +3248,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="n">
         <v>1</v>
       </c>
@@ -3233,7 +3273,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="n">
         <v>9</v>
       </c>
@@ -3258,7 +3298,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="n">
         <v>1</v>
       </c>
@@ -3283,7 +3323,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="n">
         <v>11</v>
       </c>
@@ -3308,7 +3348,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="n">
         <v>36</v>
       </c>
@@ -3333,7 +3373,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="n">
         <v>1</v>
       </c>
@@ -3364,7 +3404,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="n">
         <v>1</v>
       </c>
@@ -3395,7 +3435,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="n">
         <v>1</v>
       </c>
@@ -3426,7 +3466,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="n">
         <v>22</v>
       </c>
@@ -3451,7 +3491,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="n">
         <v>21</v>
       </c>
@@ -3476,7 +3516,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="n">
         <v>20</v>
       </c>
@@ -3501,7 +3541,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="n">
         <v>18</v>
       </c>
@@ -3526,7 +3566,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="n">
         <v>19</v>
       </c>
@@ -3551,7 +3591,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="n">
         <v>1</v>
       </c>
@@ -3584,7 +3624,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="n">
         <v>1</v>
       </c>
@@ -3615,7 +3655,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="n">
         <v>23</v>
       </c>
@@ -3640,7 +3680,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="n">
         <v>24</v>
       </c>
@@ -3690,7 +3730,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="n">
         <v>1</v>
       </c>
@@ -3721,7 +3761,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="n">
         <v>1</v>
       </c>
@@ -3752,7 +3792,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="n">
         <v>38</v>
       </c>
@@ -3777,7 +3817,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="n">
         <v>23</v>
       </c>
@@ -3974,7 +4014,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="n">
         <v>1</v>
       </c>
@@ -4005,7 +4045,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="n">
         <v>24</v>
       </c>
@@ -4030,7 +4070,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="n">
         <v>29</v>
       </c>
@@ -4080,7 +4120,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="n">
         <v>34</v>
       </c>
@@ -4105,7 +4145,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="n">
         <v>32</v>
       </c>
@@ -4180,7 +4220,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="n">
         <v>1</v>
       </c>
@@ -4205,7 +4245,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="n">
         <v>28</v>
       </c>
@@ -4255,7 +4295,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="n">
         <v>30</v>
       </c>
@@ -4280,7 +4320,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="n">
         <v>1</v>
       </c>
@@ -4336,7 +4376,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="n">
         <v>27</v>
       </c>
@@ -4361,7 +4401,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="n">
         <v>27</v>
       </c>
@@ -4386,7 +4426,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="n">
         <v>27</v>
       </c>
@@ -4411,7 +4451,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="n">
         <v>4</v>
       </c>
@@ -4436,7 +4476,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="n">
         <v>27</v>
       </c>
@@ -4461,7 +4501,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="n">
         <v>27</v>
       </c>
@@ -4486,7 +4526,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="n">
         <v>27</v>
       </c>
@@ -4511,7 +4551,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="n">
         <v>35</v>
       </c>
@@ -4536,7 +4576,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="n">
         <v>1</v>
       </c>
@@ -4586,7 +4626,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="n">
         <v>37</v>
       </c>
@@ -4611,7 +4651,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="n">
         <v>37</v>
       </c>
@@ -4636,7 +4676,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="n">
         <v>38</v>
       </c>
@@ -4661,7 +4701,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="n">
         <v>39</v>
       </c>
@@ -4686,7 +4726,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="n">
         <v>40</v>
       </c>
@@ -4711,7 +4751,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="n">
         <v>1</v>
       </c>
@@ -4736,7 +4776,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="5" t="n">
         <v>37</v>
       </c>
@@ -4761,7 +4801,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="n">
         <v>41</v>
       </c>
@@ -4786,7 +4826,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="5" t="n">
         <v>37</v>
       </c>
@@ -4811,7 +4851,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="n">
         <v>37</v>
       </c>
@@ -4836,7 +4876,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="n">
         <v>43</v>
       </c>
@@ -4861,7 +4901,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="5" t="n">
         <v>42</v>
       </c>
@@ -4886,7 +4926,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="5" t="n">
         <v>3</v>
       </c>
@@ -4911,7 +4951,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="5" t="n">
         <v>37</v>
       </c>
@@ -4936,7 +4976,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="5" t="n">
         <v>37</v>
       </c>
@@ -4961,7 +5001,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="5" t="n">
         <v>37</v>
       </c>
@@ -4986,7 +5026,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="5" t="n">
         <v>37</v>
       </c>
@@ -5011,7 +5051,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="5" t="n">
         <v>3</v>
       </c>
@@ -5036,7 +5076,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="5" t="n">
         <v>48</v>
       </c>
@@ -5061,7 +5101,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="5" t="n">
         <v>1</v>
       </c>
@@ -5086,7 +5126,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="5" t="n">
         <v>37</v>
       </c>
@@ -5111,7 +5151,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="5" t="n">
         <v>49</v>
       </c>
@@ -5136,7 +5176,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="5" t="n">
         <v>37</v>
       </c>
@@ -5161,7 +5201,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="5" t="n">
         <v>37</v>
       </c>
@@ -5279,7 +5319,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="5" t="n">
         <v>55</v>
       </c>
@@ -5304,7 +5344,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="5" t="n">
         <v>54</v>
       </c>
@@ -5329,7 +5369,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="5" t="n">
         <v>53</v>
       </c>
@@ -5354,7 +5394,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="5" t="n">
         <v>52</v>
       </c>
@@ -5379,7 +5419,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="5" t="n">
         <v>51</v>
       </c>
@@ -5404,7 +5444,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="5" t="n">
         <v>32</v>
       </c>
@@ -5429,7 +5469,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="5" t="n">
         <v>59</v>
       </c>
@@ -5454,7 +5494,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="5" t="n">
         <v>61</v>
       </c>
@@ -5479,7 +5519,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="5" t="n">
         <v>62</v>
       </c>
@@ -5504,7 +5544,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="5" t="n">
         <v>63</v>
       </c>
@@ -5529,7 +5569,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="5" t="n">
         <v>37</v>
       </c>
@@ -5554,7 +5594,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="5" t="n">
         <v>1</v>
       </c>
@@ -5579,7 +5619,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="5" t="n">
         <v>64</v>
       </c>
@@ -5604,7 +5644,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="5" t="n">
         <v>66</v>
       </c>
@@ -5629,7 +5669,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="5" t="n">
         <v>17</v>
       </c>
@@ -5754,7 +5794,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="5" t="n">
         <v>18</v>
       </c>
@@ -5779,7 +5819,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="5" t="n">
         <v>1</v>
       </c>
@@ -5810,7 +5850,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="5" t="n">
         <v>29</v>
       </c>
@@ -5860,7 +5900,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="5" t="n">
         <v>24</v>
       </c>
@@ -5885,7 +5925,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="5" t="n">
         <v>25</v>
       </c>
@@ -5941,7 +5981,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="121" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="121" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="5" t="n">
         <v>1</v>
       </c>
@@ -5972,7 +6012,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="122" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="122" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="5" t="n">
         <v>34</v>
       </c>
@@ -5997,7 +6037,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="18" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="5" t="n">
         <v>32</v>
       </c>
@@ -9825,7 +9865,9 @@
       <c r="D254" s="5" t="s">
         <v>581</v>
       </c>
-      <c r="E254" s="5"/>
+      <c r="E254" s="8" t="s">
+        <v>41</v>
+      </c>
       <c r="F254" s="6"/>
       <c r="G254" s="6"/>
       <c r="H254" s="6"/>
@@ -11214,29 +11256,30 @@
       </c>
     </row>
     <row r="308" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A308" s="8" t="s">
+      <c r="A308" s="9" t="s">
         <v>693</v>
       </c>
     </row>
     <row r="309" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A309" s="9"/>
-      <c r="B309" s="10" t="s">
+      <c r="A309" s="10"/>
+      <c r="B309" s="11" t="s">
         <v>694</v>
       </c>
     </row>
     <row r="310" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A310" s="11"/>
-      <c r="B310" s="10" t="s">
+      <c r="A310" s="12"/>
+      <c r="B310" s="11" t="s">
         <v>695</v>
       </c>
     </row>
     <row r="311" customFormat="false" ht="21.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A311" s="12"/>
-      <c r="B311" s="10" t="s">
+      <c r="A311" s="13"/>
+      <c r="B311" s="11" t="s">
         <v>696</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K306"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -11244,6 +11287,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -11264,177 +11308,177 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="14" t="s">
         <v>698</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="14" t="s">
         <v>699</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="14" t="s">
         <v>700</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="14" t="s">
         <v>701</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="14" t="s">
         <v>702</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="14" t="s">
         <v>703</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="14" t="s">
         <v>704</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="14" t="s">
         <v>705</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="14" t="s">
         <v>706</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="14" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="14" t="s">
         <v>708</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="14" t="s">
         <v>709</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="14" t="s">
         <v>710</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="14" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="14" t="s">
         <v>711</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="14" t="s">
         <v>712</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="14" t="s">
         <v>713</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
+      <c r="A19" s="14" t="s">
         <v>714</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="14" t="s">
         <v>715</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="14" t="s">
         <v>716</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="14" t="s">
         <v>717</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="14" t="s">
         <v>718</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="14" t="s">
         <v>719</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="14" t="s">
         <v>720</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
+      <c r="A26" s="14" t="s">
         <v>721</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="14" t="s">
         <v>722</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="s">
+      <c r="A28" s="14" t="s">
         <v>723</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="14" t="s">
         <v>724</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13" t="s">
+      <c r="A30" s="14" t="s">
         <v>725</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="13" t="s">
+      <c r="A31" s="14" t="s">
         <v>726</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="13" t="s">
+      <c r="A32" s="14" t="s">
         <v>727</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="13" t="s">
+      <c r="A33" s="14" t="s">
         <v>728</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="13" t="s">
+      <c r="A34" s="14" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="13" t="s">
+      <c r="A35" s="14" t="s">
         <v>729</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="13" t="s">
+      <c r="A36" s="14" t="s">
         <v>730</v>
       </c>
     </row>
@@ -11463,12 +11507,12 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>731</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -11485,100 +11529,100 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="14" t="s">
         <v>736</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="14" t="s">
         <v>737</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="16" t="s">
         <v>738</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="14" t="s">
         <v>739</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="14" t="s">
         <v>740</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="14" t="s">
         <v>741</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="14" t="s">
         <v>742</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="14" t="s">
         <v>743</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="14" t="s">
         <v>744</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="14" t="s">
         <v>745</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>743</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="14" t="s">
         <v>746</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="14" t="s">
         <v>747</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="14" t="s">
         <v>743</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="14" t="s">
         <v>748</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="14" t="s">
         <v>749</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="47.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="14" t="s">
         <v>743</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="14" t="s">
         <v>750</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="14" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="14" t="s">
         <v>737</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="14" t="s">
         <v>751</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="14" t="s">
         <v>752</v>
       </c>
     </row>

</xml_diff>